<commit_message>
Evento #1 registrado en reporte_2026-06-22.xlsx
</commit_message>
<xml_diff>
--- a/datos/excel/reporte_2026-06-22.xlsx
+++ b/datos/excel/reporte_2026-06-22.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,51 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>19:26:11</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>129</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>375</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-19.35</v>
+      </c>
+      <c r="G3" t="n">
+        <v>70</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>726.6 Hz | 1093.8 Hz | 1460.9 Hz</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>2525</v>
+      </c>
+      <c r="J3" t="n">
+        <v>11423</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>🚨 SÍ</t>
         </is>
       </c>
     </row>

</xml_diff>